<commit_message>
build: add lista_espera sheet to spreadsheet template
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/autoescuela-malaga/autoescuela_demo.xlsx
+++ b/clients/autoescuela-malaga/autoescuela_demo.xlsx
@@ -10,6 +10,7 @@
     <sheet name="agenda" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="disponibilidad" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="lista_espera" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -922,4 +923,86 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>alumno_nombre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>alumno_telefono</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>horario_preferido</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>prioridad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ana Martin</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>+34600999000</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>manana</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Diego Fernandez</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>+34600111333</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>cualquiera</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>